<commit_message>
Read classifications from CT, scope from domain reference, archive March analysis
- Instrument class from codelist NCI Preferred Term (ARCI-49 -> QS; FAQ01, FAQNA1 -> RS)
- Domain codes via CT C66734 (GASTRO -> GI, INTEGU -> IG); Physical Properties cross-domain
- COSMoS coverage joined on TESTCD + NCIt code (MCH in MB, MV in MK)
- Consumer scope from SDTM_Domain_Metadata; RE and EG in Measurement_Findings
- Ten domains added from C66734 (class only); new Scope_Check release gate
- Full refresh re-run; Changes_2026-10.md; update box on Changes_2026-09.md
- Behavioural analysis and domain overview archived (docs/archive/behavioural-analysis-2026-03/)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ndgbpomxbp7qzdpv1ucjv
</commit_message>
<xml_diff>
--- a/link-semantics/interim/Link_Kind_Audit.xlsx
+++ b/link-semantics/interim/Link_Kind_Audit.xlsx
@@ -11911,7 +11911,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>c8ef6279d51d7f5e293c0d4984336aeda8f6d3b8</t>
+          <t>c3549da46c92a9ff191f6ccb46706922955bebfd</t>
         </is>
       </c>
     </row>
@@ -11971,7 +11971,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-30 18:19:16</t>
+          <t>2026-10-01 10:39:19</t>
         </is>
       </c>
     </row>
@@ -11983,7 +11983,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-30 18:19:26</t>
+          <t>2026-10-01 10:39:28</t>
         </is>
       </c>
     </row>
@@ -11995,7 +11995,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-30 18:19</t>
+          <t>2026-10-01 10:39</t>
         </is>
       </c>
     </row>

</xml_diff>